<commit_message>
Fix YoY join bug and wire STABLE_TOLERANCE_PCT into variance status
</commit_message>
<xml_diff>
--- a/sample_output/variance_report.xlsx
+++ b/sample_output/variance_report.xlsx
@@ -879,13 +879,13 @@
         <v>0.0071</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>69477.53</v>
+        <v>68483.50999999999</v>
       </c>
       <c r="I2" s="4" t="n">
-        <v>6058.06</v>
+        <v>7052.08</v>
       </c>
       <c r="J2" s="5" t="n">
-        <v>0.0872</v>
+        <v>0.103</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
@@ -894,7 +894,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Deviation</t>
+          <t>On Plan</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -932,13 +932,13 @@
         <v>-0.0395</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>53126.43</v>
+        <v>57727.97</v>
       </c>
       <c r="I3" s="4" t="n">
-        <v>4504.76</v>
+        <v>-96.78</v>
       </c>
       <c r="J3" s="5" t="n">
-        <v>0.0848</v>
+        <v>-0.0017</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
@@ -985,13 +985,13 @@
         <v>0.0248</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>40524.85</v>
+        <v>40058.17</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>5589.1</v>
+        <v>6055.78</v>
       </c>
       <c r="J4" s="5" t="n">
-        <v>0.1379</v>
+        <v>0.1512</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
@@ -1038,13 +1038,13 @@
         <v>0.0141</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>194684.62</v>
+        <v>184066.34</v>
       </c>
       <c r="I5" s="4" t="n">
-        <v>17269.8</v>
+        <v>27888.08</v>
       </c>
       <c r="J5" s="5" t="n">
-        <v>0.08869999999999999</v>
+        <v>0.1515</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
@@ -1091,13 +1091,13 @@
         <v>0.0314</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>133213.11</v>
+        <v>129978.32</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>13757.74</v>
+        <v>16992.53</v>
       </c>
       <c r="J6" s="5" t="n">
-        <v>0.1033</v>
+        <v>0.1307</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
@@ -1144,13 +1144,13 @@
         <v>0.0189</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>251763.73</v>
+        <v>253278.78</v>
       </c>
       <c r="I7" s="4" t="n">
-        <v>19268.38</v>
+        <v>17753.33</v>
       </c>
       <c r="J7" s="5" t="n">
-        <v>0.0765</v>
+        <v>0.0701</v>
       </c>
       <c r="K7" t="inlineStr">
         <is>
@@ -1197,13 +1197,13 @@
         <v>-0.033</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>72952.21000000001</v>
+        <v>70827.32000000001</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>536.38</v>
+        <v>2661.27</v>
       </c>
       <c r="J8" s="5" t="n">
-        <v>0.0074</v>
+        <v>0.03759999999999999</v>
       </c>
       <c r="K8" t="inlineStr">
         <is>
@@ -1250,13 +1250,13 @@
         <v>-0.0357</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="I9" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J9" s="5" t="n">
-        <v>0.08</v>
+        <v>0.125</v>
       </c>
       <c r="K9" t="inlineStr">
         <is>
@@ -1275,7 +1275,7 @@
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>Engineering headcount was 1 below plan in January 2024. This is a deviation from plan, flagged for routine review. Compared to the same period last year, this is up 8.0%.</t>
+          <t>Engineering headcount was 1 below plan in January 2024. This is a deviation from plan, flagged for routine review. Compared to the same period last year, this is up 12.5%.</t>
         </is>
       </c>
     </row>
@@ -1361,13 +1361,13 @@
         <v>0</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="I11" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J11" s="5" t="n">
-        <v>0.1538</v>
+        <v>0.07139999999999999</v>
       </c>
       <c r="K11" t="inlineStr">
         <is>
@@ -1414,13 +1414,13 @@
         <v>0</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="I12" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J12" s="5" t="n">
-        <v>0</v>
+        <v>0.1429</v>
       </c>
       <c r="K12" t="inlineStr">
         <is>
@@ -1467,13 +1467,13 @@
         <v>-0.03759999999999999</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>105347.37</v>
+        <v>106939.36</v>
       </c>
       <c r="I13" s="4" t="n">
-        <v>4364.38</v>
+        <v>2772.39</v>
       </c>
       <c r="J13" s="5" t="n">
-        <v>0.0414</v>
+        <v>0.0259</v>
       </c>
       <c r="K13" t="inlineStr">
         <is>
@@ -1520,13 +1520,13 @@
         <v>-0.0379</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>54152.85</v>
+        <v>53258.37</v>
       </c>
       <c r="I14" s="4" t="n">
-        <v>688.15</v>
+        <v>1582.63</v>
       </c>
       <c r="J14" s="5" t="n">
-        <v>0.0127</v>
+        <v>0.0297</v>
       </c>
       <c r="K14" t="inlineStr">
         <is>
@@ -1573,13 +1573,13 @@
         <v>-0.0225</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>79821.28999999999</v>
+        <v>78615.77</v>
       </c>
       <c r="I15" s="4" t="n">
-        <v>3754.19</v>
+        <v>4959.71</v>
       </c>
       <c r="J15" s="5" t="n">
-        <v>0.047</v>
+        <v>0.06309999999999999</v>
       </c>
       <c r="K15" t="inlineStr">
         <is>
@@ -1626,13 +1626,13 @@
         <v>-0.0062</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>329633.72</v>
+        <v>321971.58</v>
       </c>
       <c r="I16" s="4" t="n">
-        <v>29111.38</v>
+        <v>36773.52</v>
       </c>
       <c r="J16" s="5" t="n">
-        <v>0.0883</v>
+        <v>0.1142</v>
       </c>
       <c r="K16" t="inlineStr">
         <is>
@@ -1679,13 +1679,13 @@
         <v>0.0004</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>31839.33</v>
+        <v>29806.85</v>
       </c>
       <c r="I17" s="4" t="n">
-        <v>1424.92</v>
+        <v>3457.4</v>
       </c>
       <c r="J17" s="5" t="n">
-        <v>0.04480000000000001</v>
+        <v>0.116</v>
       </c>
       <c r="K17" t="inlineStr">
         <is>
@@ -1732,13 +1732,13 @@
         <v>-0.0221</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>163988.97</v>
+        <v>156928.84</v>
       </c>
       <c r="I18" s="4" t="n">
-        <v>3224.55</v>
+        <v>10284.68</v>
       </c>
       <c r="J18" s="5" t="n">
-        <v>0.0197</v>
+        <v>0.0655</v>
       </c>
       <c r="K18" t="inlineStr">
         <is>
@@ -1785,13 +1785,13 @@
         <v>0.0112</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>713392.89</v>
+        <v>678163.16</v>
       </c>
       <c r="I19" s="4" t="n">
-        <v>55084.26</v>
+        <v>90313.99000000001</v>
       </c>
       <c r="J19" s="5" t="n">
-        <v>0.07719999999999999</v>
+        <v>0.1332</v>
       </c>
       <c r="K19" t="inlineStr">
         <is>
@@ -1838,13 +1838,13 @@
         <v>-0.038</v>
       </c>
       <c r="H20" s="4" t="n">
-        <v>391492.05</v>
+        <v>374595.65</v>
       </c>
       <c r="I20" s="4" t="n">
-        <v>19763.32</v>
+        <v>36659.72</v>
       </c>
       <c r="J20" s="5" t="n">
-        <v>0.0505</v>
+        <v>0.09789999999999999</v>
       </c>
       <c r="K20" t="inlineStr">
         <is>
@@ -1891,13 +1891,13 @@
         <v>-0.018</v>
       </c>
       <c r="H21" s="4" t="n">
-        <v>284920.78</v>
+        <v>272543.76</v>
       </c>
       <c r="I21" s="4" t="n">
-        <v>13607.93</v>
+        <v>25984.95</v>
       </c>
       <c r="J21" s="5" t="n">
-        <v>0.0478</v>
+        <v>0.0953</v>
       </c>
       <c r="K21" t="inlineStr">
         <is>
@@ -1944,13 +1944,13 @@
         <v>-0.0128</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>365075.96</v>
+        <v>340831.97</v>
       </c>
       <c r="I22" s="4" t="n">
-        <v>10067.66</v>
+        <v>34311.65</v>
       </c>
       <c r="J22" s="5" t="n">
-        <v>0.0276</v>
+        <v>0.1007</v>
       </c>
       <c r="K22" t="inlineStr">
         <is>
@@ -1959,7 +1959,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>Deviation</t>
+          <t>On Plan</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
@@ -1997,13 +1997,13 @@
         <v>0.0159</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>394117.71</v>
+        <v>369020.44</v>
       </c>
       <c r="I23" s="4" t="n">
-        <v>32539.77</v>
+        <v>57637.04</v>
       </c>
       <c r="J23" s="5" t="n">
-        <v>0.08259999999999999</v>
+        <v>0.1562</v>
       </c>
       <c r="K23" t="inlineStr">
         <is>
@@ -2012,7 +2012,7 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>Deviation</t>
+          <t>On Plan</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
@@ -2050,13 +2050,13 @@
         <v>0.0245</v>
       </c>
       <c r="H24" s="4" t="n">
-        <v>890490.46</v>
+        <v>875569.51</v>
       </c>
       <c r="I24" s="4" t="n">
-        <v>82751.8</v>
+        <v>97672.75</v>
       </c>
       <c r="J24" s="5" t="n">
-        <v>0.0929</v>
+        <v>0.1116</v>
       </c>
       <c r="K24" t="inlineStr">
         <is>
@@ -2103,13 +2103,13 @@
         <v>0.0164</v>
       </c>
       <c r="H25" s="4" t="n">
-        <v>68796.46000000001</v>
+        <v>67255.95</v>
       </c>
       <c r="I25" s="4" t="n">
-        <v>7812.11</v>
+        <v>9352.620000000001</v>
       </c>
       <c r="J25" s="5" t="n">
-        <v>0.1136</v>
+        <v>0.1391</v>
       </c>
       <c r="K25" t="inlineStr">
         <is>
@@ -2118,7 +2118,7 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>Deviation</t>
+          <t>On Plan</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
@@ -2156,13 +2156,13 @@
         <v>-0.0218</v>
       </c>
       <c r="H26" s="4" t="n">
-        <v>57496.72</v>
+        <v>56667.29</v>
       </c>
       <c r="I26" s="4" t="n">
-        <v>1490.66</v>
+        <v>2320.09</v>
       </c>
       <c r="J26" s="5" t="n">
-        <v>0.0259</v>
+        <v>0.0409</v>
       </c>
       <c r="K26" t="inlineStr">
         <is>
@@ -2209,13 +2209,13 @@
         <v>-0.0363</v>
       </c>
       <c r="H27" s="4" t="n">
-        <v>42027.25</v>
+        <v>41969.92</v>
       </c>
       <c r="I27" s="4" t="n">
-        <v>1554.54</v>
+        <v>1611.87</v>
       </c>
       <c r="J27" s="5" t="n">
-        <v>0.03700000000000001</v>
+        <v>0.0384</v>
       </c>
       <c r="K27" t="inlineStr">
         <is>
@@ -2262,13 +2262,13 @@
         <v>0.0278</v>
       </c>
       <c r="H28" s="4" t="n">
-        <v>182899.49</v>
+        <v>187985.4</v>
       </c>
       <c r="I28" s="4" t="n">
-        <v>26167.27</v>
+        <v>21081.36</v>
       </c>
       <c r="J28" s="5" t="n">
-        <v>0.1431</v>
+        <v>0.1121</v>
       </c>
       <c r="K28" t="inlineStr">
         <is>
@@ -2315,13 +2315,13 @@
         <v>0.0083</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>123790.67</v>
+        <v>132673.7</v>
       </c>
       <c r="I29" s="4" t="n">
-        <v>16050.19</v>
+        <v>7167.16</v>
       </c>
       <c r="J29" s="5" t="n">
-        <v>0.1297</v>
+        <v>0.05400000000000001</v>
       </c>
       <c r="K29" t="inlineStr">
         <is>
@@ -2368,13 +2368,13 @@
         <v>-0.0323</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>235381.13</v>
+        <v>248554.66</v>
       </c>
       <c r="I30" s="4" t="n">
-        <v>15154.45</v>
+        <v>1980.92</v>
       </c>
       <c r="J30" s="5" t="n">
-        <v>0.0644</v>
+        <v>0.008</v>
       </c>
       <c r="K30" t="inlineStr">
         <is>
@@ -2421,13 +2421,13 @@
         <v>0.0246</v>
       </c>
       <c r="H31" s="4" t="n">
-        <v>64944.79</v>
+        <v>70362.42</v>
       </c>
       <c r="I31" s="4" t="n">
-        <v>10840.62</v>
+        <v>5422.99</v>
       </c>
       <c r="J31" s="5" t="n">
-        <v>0.1669</v>
+        <v>0.0771</v>
       </c>
       <c r="K31" t="inlineStr">
         <is>
@@ -2474,13 +2474,13 @@
         <v>0.0357</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="I32" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J32" s="5" t="n">
-        <v>0.1154</v>
+        <v>0.0741</v>
       </c>
       <c r="K32" t="inlineStr">
         <is>
@@ -2499,7 +2499,7 @@
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>Engineering headcount was 1 above plan in February 2024. This is a deviation from plan, flagged for routine review. Compared to the same period last year, this is up 11.5%.</t>
+          <t>Engineering headcount was 1 above plan in February 2024. This is a deviation from plan, flagged for routine review. Compared to the same period last year, this is up 7.4%.</t>
         </is>
       </c>
     </row>
@@ -2585,13 +2585,13 @@
         <v>0</v>
       </c>
       <c r="H34" s="4" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="I34" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J34" s="5" t="n">
-        <v>0.1538</v>
+        <v>0.07139999999999999</v>
       </c>
       <c r="K34" t="inlineStr">
         <is>
@@ -2638,13 +2638,13 @@
         <v>0</v>
       </c>
       <c r="H35" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="I35" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J35" s="5" t="n">
-        <v>0</v>
+        <v>0.1429</v>
       </c>
       <c r="K35" t="inlineStr">
         <is>
@@ -2691,13 +2691,13 @@
         <v>0.0029</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>104980.26</v>
+        <v>103795.12</v>
       </c>
       <c r="I36" s="4" t="n">
-        <v>6293.31</v>
+        <v>7478.45</v>
       </c>
       <c r="J36" s="5" t="n">
-        <v>0.0599</v>
+        <v>0.0721</v>
       </c>
       <c r="K36" t="inlineStr">
         <is>
@@ -2744,13 +2744,13 @@
         <v>0.0042</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>53321.03</v>
+        <v>51027.11</v>
       </c>
       <c r="I37" s="4" t="n">
-        <v>2385.93</v>
+        <v>4679.85</v>
       </c>
       <c r="J37" s="5" t="n">
-        <v>0.0447</v>
+        <v>0.0917</v>
       </c>
       <c r="K37" t="inlineStr">
         <is>
@@ -2797,13 +2797,13 @@
         <v>0.0378</v>
       </c>
       <c r="H38" s="4" t="n">
-        <v>76748.84</v>
+        <v>76212.39999999999</v>
       </c>
       <c r="I38" s="4" t="n">
-        <v>9614.75</v>
+        <v>10151.19</v>
       </c>
       <c r="J38" s="5" t="n">
-        <v>0.1253</v>
+        <v>0.1332</v>
       </c>
       <c r="K38" t="inlineStr">
         <is>
@@ -2850,13 +2850,13 @@
         <v>0.0184</v>
       </c>
       <c r="H39" s="4" t="n">
-        <v>336488.54</v>
+        <v>325255.26</v>
       </c>
       <c r="I39" s="4" t="n">
-        <v>21316.72</v>
+        <v>32550</v>
       </c>
       <c r="J39" s="5" t="n">
-        <v>0.0634</v>
+        <v>0.1001</v>
       </c>
       <c r="K39" t="inlineStr">
         <is>
@@ -2903,13 +2903,13 @@
         <v>-0.0097</v>
       </c>
       <c r="H40" s="4" t="n">
-        <v>30959.41</v>
+        <v>30603.28</v>
       </c>
       <c r="I40" s="4" t="n">
-        <v>1087.13</v>
+        <v>1443.26</v>
       </c>
       <c r="J40" s="5" t="n">
-        <v>0.0351</v>
+        <v>0.0472</v>
       </c>
       <c r="K40" t="inlineStr">
         <is>
@@ -2956,13 +2956,13 @@
         <v>-0.0326</v>
       </c>
       <c r="H41" s="4" t="n">
-        <v>145341.69</v>
+        <v>154905.08</v>
       </c>
       <c r="I41" s="4" t="n">
-        <v>15664.03</v>
+        <v>6100.64</v>
       </c>
       <c r="J41" s="5" t="n">
-        <v>0.1078</v>
+        <v>0.0394</v>
       </c>
       <c r="K41" t="inlineStr">
         <is>
@@ -3009,13 +3009,13 @@
         <v>-0.0276</v>
       </c>
       <c r="H42" s="4" t="n">
-        <v>677151.97</v>
+        <v>700706.55</v>
       </c>
       <c r="I42" s="4" t="n">
-        <v>42141.24</v>
+        <v>18586.66</v>
       </c>
       <c r="J42" s="5" t="n">
-        <v>0.0622</v>
+        <v>0.0265</v>
       </c>
       <c r="K42" t="inlineStr">
         <is>
@@ -3062,13 +3062,13 @@
         <v>0.0366</v>
       </c>
       <c r="H43" s="4" t="n">
-        <v>380643.67</v>
+        <v>379221.72</v>
       </c>
       <c r="I43" s="4" t="n">
-        <v>50644.94</v>
+        <v>52066.89</v>
       </c>
       <c r="J43" s="5" t="n">
-        <v>0.1331</v>
+        <v>0.1373</v>
       </c>
       <c r="K43" t="inlineStr">
         <is>
@@ -3115,13 +3115,13 @@
         <v>-0.0131</v>
       </c>
       <c r="H44" s="4" t="n">
-        <v>259484.35</v>
+        <v>279011.81</v>
       </c>
       <c r="I44" s="4" t="n">
-        <v>32519.88</v>
+        <v>12992.42</v>
       </c>
       <c r="J44" s="5" t="n">
-        <v>0.1253</v>
+        <v>0.0466</v>
       </c>
       <c r="K44" t="inlineStr">
         <is>
@@ -3168,13 +3168,13 @@
         <v>-0.0214</v>
       </c>
       <c r="H45" s="4" t="n">
-        <v>354312.07</v>
+        <v>341719.93</v>
       </c>
       <c r="I45" s="4" t="n">
-        <v>19424.16</v>
+        <v>32016.3</v>
       </c>
       <c r="J45" s="5" t="n">
-        <v>0.0548</v>
+        <v>0.09369999999999999</v>
       </c>
       <c r="K45" t="inlineStr">
         <is>
@@ -3221,13 +3221,13 @@
         <v>-0.0336</v>
       </c>
       <c r="H46" s="4" t="n">
-        <v>389697.14</v>
+        <v>391297.56</v>
       </c>
       <c r="I46" s="4" t="n">
-        <v>18213.28</v>
+        <v>16612.86</v>
       </c>
       <c r="J46" s="5" t="n">
-        <v>0.0467</v>
+        <v>0.0425</v>
       </c>
       <c r="K46" t="inlineStr">
         <is>
@@ -3274,13 +3274,13 @@
         <v>-0.0168</v>
       </c>
       <c r="H47" s="4" t="n">
-        <v>846162.15</v>
+        <v>875861.6</v>
       </c>
       <c r="I47" s="4" t="n">
-        <v>92501.3</v>
+        <v>62801.85</v>
       </c>
       <c r="J47" s="5" t="n">
-        <v>0.1093</v>
+        <v>0.0717</v>
       </c>
       <c r="K47" t="inlineStr">
         <is>
@@ -3289,7 +3289,7 @@
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>Deviation</t>
+          <t>On Plan</t>
         </is>
       </c>
       <c r="M47" t="inlineStr">
@@ -3327,13 +3327,13 @@
         <v>0.0148</v>
       </c>
       <c r="H48" s="4" t="n">
-        <v>69100.71000000001</v>
+        <v>70349.11</v>
       </c>
       <c r="I48" s="4" t="n">
-        <v>7768.05</v>
+        <v>6519.65</v>
       </c>
       <c r="J48" s="5" t="n">
-        <v>0.1124</v>
+        <v>0.09269999999999999</v>
       </c>
       <c r="K48" t="inlineStr">
         <is>
@@ -3342,7 +3342,7 @@
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>Deviation</t>
+          <t>On Plan</t>
         </is>
       </c>
       <c r="M48" t="inlineStr">
@@ -3380,13 +3380,13 @@
         <v>0.0221</v>
       </c>
       <c r="H49" s="4" t="n">
-        <v>56070.29</v>
+        <v>56666.08</v>
       </c>
       <c r="I49" s="4" t="n">
-        <v>5867.76</v>
+        <v>5271.97</v>
       </c>
       <c r="J49" s="5" t="n">
-        <v>0.1047</v>
+        <v>0.09300000000000001</v>
       </c>
       <c r="K49" t="inlineStr">
         <is>
@@ -3433,13 +3433,13 @@
         <v>0.0274</v>
       </c>
       <c r="H50" s="4" t="n">
-        <v>43420.81</v>
+        <v>42876.87</v>
       </c>
       <c r="I50" s="4" t="n">
-        <v>3275.8</v>
+        <v>3819.74</v>
       </c>
       <c r="J50" s="5" t="n">
-        <v>0.07539999999999999</v>
+        <v>0.0891</v>
       </c>
       <c r="K50" t="inlineStr">
         <is>
@@ -3486,13 +3486,13 @@
         <v>-0.0232</v>
       </c>
       <c r="H51" s="4" t="n">
-        <v>213833.33</v>
+        <v>198982.3</v>
       </c>
       <c r="I51" s="4" t="n">
-        <v>7543.59</v>
+        <v>22394.62</v>
       </c>
       <c r="J51" s="5" t="n">
-        <v>0.0353</v>
+        <v>0.1125</v>
       </c>
       <c r="K51" t="inlineStr">
         <is>
@@ -3539,13 +3539,13 @@
         <v>-0.0186</v>
       </c>
       <c r="H52" s="4" t="n">
-        <v>138364.32</v>
+        <v>136977.24</v>
       </c>
       <c r="I52" s="4" t="n">
-        <v>13284.97</v>
+        <v>14672.05</v>
       </c>
       <c r="J52" s="5" t="n">
-        <v>0.096</v>
+        <v>0.1071</v>
       </c>
       <c r="K52" t="inlineStr">
         <is>
@@ -3592,13 +3592,13 @@
         <v>-0.0104</v>
       </c>
       <c r="H53" s="4" t="n">
-        <v>267222.29</v>
+        <v>263807.01</v>
       </c>
       <c r="I53" s="4" t="n">
-        <v>18237.94</v>
+        <v>21653.22</v>
       </c>
       <c r="J53" s="5" t="n">
-        <v>0.0683</v>
+        <v>0.08210000000000001</v>
       </c>
       <c r="K53" t="inlineStr">
         <is>
@@ -3645,10 +3645,10 @@
         <v>0.0349</v>
       </c>
       <c r="H54" s="4" t="n">
-        <v>76525.95</v>
+        <v>76528.02</v>
       </c>
       <c r="I54" s="4" t="n">
-        <v>8769.040000000001</v>
+        <v>8766.969999999999</v>
       </c>
       <c r="J54" s="5" t="n">
         <v>0.1146</v>
@@ -3751,13 +3751,13 @@
         <v>0</v>
       </c>
       <c r="H56" s="4" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="I56" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J56" s="5" t="n">
-        <v>0</v>
+        <v>0.09089999999999999</v>
       </c>
       <c r="K56" t="inlineStr">
         <is>
@@ -3915,13 +3915,13 @@
         <v>0.008699999999999999</v>
       </c>
       <c r="H59" s="4" t="n">
-        <v>117621.24</v>
+        <v>107700.87</v>
       </c>
       <c r="I59" s="4" t="n">
-        <v>7082.06</v>
+        <v>17002.43</v>
       </c>
       <c r="J59" s="5" t="n">
-        <v>0.0602</v>
+        <v>0.1579</v>
       </c>
       <c r="K59" t="inlineStr">
         <is>
@@ -3968,13 +3968,13 @@
         <v>-0.0269</v>
       </c>
       <c r="H60" s="4" t="n">
-        <v>56049.65</v>
+        <v>55829.78</v>
       </c>
       <c r="I60" s="4" t="n">
-        <v>4097.89</v>
+        <v>4317.76</v>
       </c>
       <c r="J60" s="5" t="n">
-        <v>0.0731</v>
+        <v>0.07730000000000001</v>
       </c>
       <c r="K60" t="inlineStr">
         <is>
@@ -4021,13 +4021,13 @@
         <v>-0.0263</v>
       </c>
       <c r="H61" s="4" t="n">
-        <v>87104.25</v>
+        <v>83675.62</v>
       </c>
       <c r="I61" s="4" t="n">
-        <v>3174.44</v>
+        <v>6603.07</v>
       </c>
       <c r="J61" s="5" t="n">
-        <v>0.0364</v>
+        <v>0.0789</v>
       </c>
       <c r="K61" t="inlineStr">
         <is>
@@ -4074,13 +4074,13 @@
         <v>0.0118</v>
       </c>
       <c r="H62" s="4" t="n">
-        <v>349040.02</v>
+        <v>363952.74</v>
       </c>
       <c r="I62" s="4" t="n">
-        <v>47072.16</v>
+        <v>32159.44</v>
       </c>
       <c r="J62" s="5" t="n">
-        <v>0.1349</v>
+        <v>0.08839999999999999</v>
       </c>
       <c r="K62" t="inlineStr">
         <is>
@@ -4127,13 +4127,13 @@
         <v>0.0183</v>
       </c>
       <c r="H63" s="4" t="n">
-        <v>33008.54</v>
+        <v>32983.95</v>
       </c>
       <c r="I63" s="4" t="n">
-        <v>3709.39</v>
+        <v>3733.98</v>
       </c>
       <c r="J63" s="5" t="n">
-        <v>0.1124</v>
+        <v>0.1132</v>
       </c>
       <c r="K63" t="inlineStr">
         <is>
@@ -4180,13 +4180,13 @@
         <v>-0.0108</v>
       </c>
       <c r="H64" s="4" t="n">
-        <v>166096.38</v>
+        <v>165866.68</v>
       </c>
       <c r="I64" s="4" t="n">
-        <v>17334.42</v>
+        <v>17564.12</v>
       </c>
       <c r="J64" s="5" t="n">
-        <v>0.1044</v>
+        <v>0.1059</v>
       </c>
       <c r="K64" t="inlineStr">
         <is>
@@ -4233,13 +4233,13 @@
         <v>-0.0319</v>
       </c>
       <c r="H65" s="4" t="n">
-        <v>750098.84</v>
+        <v>719000.83</v>
       </c>
       <c r="I65" s="4" t="n">
-        <v>47754.07</v>
+        <v>78852.08</v>
       </c>
       <c r="J65" s="5" t="n">
-        <v>0.06370000000000001</v>
+        <v>0.1097</v>
       </c>
       <c r="K65" t="inlineStr">
         <is>
@@ -4286,13 +4286,13 @@
         <v>-0.0178</v>
       </c>
       <c r="H66" s="4" t="n">
-        <v>405018.98</v>
+        <v>413231.73</v>
       </c>
       <c r="I66" s="4" t="n">
-        <v>50336.68</v>
+        <v>42123.93</v>
       </c>
       <c r="J66" s="5" t="n">
-        <v>0.1243</v>
+        <v>0.1019</v>
       </c>
       <c r="K66" t="inlineStr">
         <is>
@@ -4339,13 +4339,13 @@
         <v>0.0109</v>
       </c>
       <c r="H67" s="4" t="n">
-        <v>295722.45</v>
+        <v>293432.88</v>
       </c>
       <c r="I67" s="4" t="n">
-        <v>37519.97</v>
+        <v>39809.54</v>
       </c>
       <c r="J67" s="5" t="n">
-        <v>0.1269</v>
+        <v>0.1357</v>
       </c>
       <c r="K67" t="inlineStr">
         <is>
@@ -4392,13 +4392,13 @@
         <v>-0.0148</v>
       </c>
       <c r="H68" s="4" t="n">
-        <v>338677.89</v>
+        <v>344417.49</v>
       </c>
       <c r="I68" s="4" t="n">
-        <v>39455.78</v>
+        <v>33716.18</v>
       </c>
       <c r="J68" s="5" t="n">
-        <v>0.1165</v>
+        <v>0.09789999999999999</v>
       </c>
       <c r="K68" t="inlineStr">
         <is>
@@ -4407,7 +4407,7 @@
       </c>
       <c r="L68" t="inlineStr">
         <is>
-          <t>Deviation</t>
+          <t>On Plan</t>
         </is>
       </c>
       <c r="M68" t="inlineStr">
@@ -4445,13 +4445,13 @@
         <v>-0.0374</v>
       </c>
       <c r="H69" s="4" t="n">
-        <v>383047.89</v>
+        <v>367307.82</v>
       </c>
       <c r="I69" s="4" t="n">
-        <v>25273.46</v>
+        <v>41013.53</v>
       </c>
       <c r="J69" s="5" t="n">
-        <v>0.066</v>
+        <v>0.1117</v>
       </c>
       <c r="K69" t="inlineStr">
         <is>
@@ -4498,13 +4498,13 @@
         <v>-0.0217</v>
       </c>
       <c r="H70" s="4" t="n">
-        <v>877722.6800000001</v>
+        <v>863545.3</v>
       </c>
       <c r="I70" s="4" t="n">
-        <v>60979.05</v>
+        <v>75156.42999999999</v>
       </c>
       <c r="J70" s="5" t="n">
-        <v>0.06950000000000001</v>
+        <v>0.08699999999999999</v>
       </c>
       <c r="K70" t="inlineStr">
         <is>
@@ -4551,13 +4551,13 @@
         <v>0.0398</v>
       </c>
       <c r="H71" s="4" t="n">
-        <v>72396.57000000001</v>
+        <v>69843.57000000001</v>
       </c>
       <c r="I71" s="4" t="n">
-        <v>6758.43</v>
+        <v>9311.43</v>
       </c>
       <c r="J71" s="5" t="n">
-        <v>0.0934</v>
+        <v>0.1333</v>
       </c>
       <c r="K71" t="inlineStr">
         <is>
@@ -4604,13 +4604,13 @@
         <v>-0.0327</v>
       </c>
       <c r="H72" s="4" t="n">
-        <v>54987.19</v>
+        <v>54614.99</v>
       </c>
       <c r="I72" s="4" t="n">
-        <v>3919.72</v>
+        <v>4291.92</v>
       </c>
       <c r="J72" s="5" t="n">
-        <v>0.0713</v>
+        <v>0.0786</v>
       </c>
       <c r="K72" t="inlineStr">
         <is>
@@ -4657,13 +4657,13 @@
         <v>0.0008</v>
       </c>
       <c r="H73" s="4" t="n">
-        <v>43109.53</v>
+        <v>39441.64</v>
       </c>
       <c r="I73" s="4" t="n">
-        <v>2600.28</v>
+        <v>6268.17</v>
       </c>
       <c r="J73" s="5" t="n">
-        <v>0.0603</v>
+        <v>0.1589</v>
       </c>
       <c r="K73" t="inlineStr">
         <is>
@@ -4672,7 +4672,7 @@
       </c>
       <c r="L73" t="inlineStr">
         <is>
-          <t>Deviation</t>
+          <t>On Plan</t>
         </is>
       </c>
       <c r="M73" t="inlineStr">
@@ -4710,13 +4710,13 @@
         <v>0.0124</v>
       </c>
       <c r="H74" s="4" t="n">
-        <v>213566.02</v>
+        <v>213500.4</v>
       </c>
       <c r="I74" s="4" t="n">
-        <v>23814.57</v>
+        <v>23880.19</v>
       </c>
       <c r="J74" s="5" t="n">
-        <v>0.1115</v>
+        <v>0.1119</v>
       </c>
       <c r="K74" t="inlineStr">
         <is>
@@ -4763,13 +4763,13 @@
         <v>-0.0083</v>
       </c>
       <c r="H75" s="4" t="n">
-        <v>151096.98</v>
+        <v>146396.13</v>
       </c>
       <c r="I75" s="4" t="n">
-        <v>7430.76</v>
+        <v>12131.61</v>
       </c>
       <c r="J75" s="5" t="n">
-        <v>0.0492</v>
+        <v>0.08289999999999999</v>
       </c>
       <c r="K75" t="inlineStr">
         <is>
@@ -4816,13 +4816,13 @@
         <v>-0.0148</v>
       </c>
       <c r="H76" s="4" t="n">
-        <v>262461.84</v>
+        <v>277174.8</v>
       </c>
       <c r="I76" s="4" t="n">
-        <v>31524</v>
+        <v>16811.04</v>
       </c>
       <c r="J76" s="5" t="n">
-        <v>0.1201</v>
+        <v>0.0607</v>
       </c>
       <c r="K76" t="inlineStr">
         <is>
@@ -4869,13 +4869,13 @@
         <v>0.0332</v>
       </c>
       <c r="H77" s="4" t="n">
-        <v>76801.75999999999</v>
+        <v>75120.32000000001</v>
       </c>
       <c r="I77" s="4" t="n">
-        <v>11285.79</v>
+        <v>12967.23</v>
       </c>
       <c r="J77" s="5" t="n">
-        <v>0.1469</v>
+        <v>0.1726</v>
       </c>
       <c r="K77" t="inlineStr">
         <is>
@@ -4922,13 +4922,13 @@
         <v>0.0357</v>
       </c>
       <c r="H78" s="4" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="I78" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J78" s="5" t="n">
-        <v>0.16</v>
+        <v>0.1154</v>
       </c>
       <c r="K78" t="inlineStr">
         <is>
@@ -4947,7 +4947,7 @@
       </c>
       <c r="N78" t="inlineStr">
         <is>
-          <t>Engineering headcount was 1 above plan in April 2024. This is a deviation from plan, flagged for routine review. Compared to the same period last year, this is up 16.0%.</t>
+          <t>Engineering headcount was 1 above plan in April 2024. This is a deviation from plan, flagged for routine review. Compared to the same period last year, this is up 11.5%.</t>
         </is>
       </c>
     </row>
@@ -5033,13 +5033,13 @@
         <v>0.0667</v>
       </c>
       <c r="H80" s="4" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="I80" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J80" s="5" t="n">
-        <v>0.1429</v>
+        <v>0.2308</v>
       </c>
       <c r="K80" t="inlineStr">
         <is>
@@ -5058,7 +5058,7 @@
       </c>
       <c r="N80" t="inlineStr">
         <is>
-          <t>Sales headcount was 1 above plan in April 2024. This is a deviation from plan, flagged for routine review. Compared to the same period last year, this is up 14.3%.</t>
+          <t>Sales headcount was 1 above plan in April 2024. This is a deviation from plan, flagged for routine review. Compared to the same period last year, this is up 23.1%.</t>
         </is>
       </c>
     </row>
@@ -5144,13 +5144,13 @@
         <v>-0.0188</v>
       </c>
       <c r="H82" s="4" t="n">
-        <v>111531.57</v>
+        <v>115176.21</v>
       </c>
       <c r="I82" s="4" t="n">
-        <v>13952.87</v>
+        <v>10308.23</v>
       </c>
       <c r="J82" s="5" t="n">
-        <v>0.1251</v>
+        <v>0.0895</v>
       </c>
       <c r="K82" t="inlineStr">
         <is>
@@ -5197,13 +5197,13 @@
         <v>-0.019</v>
       </c>
       <c r="H83" s="4" t="n">
-        <v>56448.97</v>
+        <v>58998.31</v>
       </c>
       <c r="I83" s="4" t="n">
-        <v>6282.31</v>
+        <v>3732.97</v>
       </c>
       <c r="J83" s="5" t="n">
-        <v>0.1113</v>
+        <v>0.0633</v>
       </c>
       <c r="K83" t="inlineStr">
         <is>
@@ -5250,13 +5250,13 @@
         <v>-0.0203</v>
       </c>
       <c r="H84" s="4" t="n">
-        <v>91053.53999999999</v>
+        <v>82845.34</v>
       </c>
       <c r="I84" s="4" t="n">
-        <v>2919.73</v>
+        <v>11127.93</v>
       </c>
       <c r="J84" s="5" t="n">
-        <v>0.0321</v>
+        <v>0.1343</v>
       </c>
       <c r="K84" t="inlineStr">
         <is>
@@ -5303,13 +5303,13 @@
         <v>-0.0033</v>
       </c>
       <c r="H85" s="4" t="n">
-        <v>374357.36</v>
+        <v>356780.53</v>
       </c>
       <c r="I85" s="4" t="n">
-        <v>29294.49</v>
+        <v>46871.32</v>
       </c>
       <c r="J85" s="5" t="n">
-        <v>0.07829999999999999</v>
+        <v>0.1314</v>
       </c>
       <c r="K85" t="inlineStr">
         <is>
@@ -5356,13 +5356,13 @@
         <v>0.0049</v>
       </c>
       <c r="H86" s="4" t="n">
-        <v>34178.1</v>
+        <v>33255.95</v>
       </c>
       <c r="I86" s="4" t="n">
-        <v>3306.28</v>
+        <v>4228.43</v>
       </c>
       <c r="J86" s="5" t="n">
-        <v>0.09669999999999999</v>
+        <v>0.1271</v>
       </c>
       <c r="K86" t="inlineStr">
         <is>
@@ -5409,13 +5409,13 @@
         <v>0.0301</v>
       </c>
       <c r="H87" s="4" t="n">
-        <v>178400.72</v>
+        <v>172471.94</v>
       </c>
       <c r="I87" s="4" t="n">
-        <v>19210.32</v>
+        <v>25139.1</v>
       </c>
       <c r="J87" s="5" t="n">
-        <v>0.1077</v>
+        <v>0.1458</v>
       </c>
       <c r="K87" t="inlineStr">
         <is>
@@ -5462,13 +5462,13 @@
         <v>-0.0186</v>
       </c>
       <c r="H88" s="4" t="n">
-        <v>762118.3100000001</v>
+        <v>792388.5600000001</v>
       </c>
       <c r="I88" s="4" t="n">
-        <v>74639.75999999999</v>
+        <v>44369.51</v>
       </c>
       <c r="J88" s="5" t="n">
-        <v>0.09789999999999999</v>
+        <v>0.05599999999999999</v>
       </c>
       <c r="K88" t="inlineStr">
         <is>
@@ -5515,13 +5515,13 @@
         <v>-0.0231</v>
       </c>
       <c r="H89" s="4" t="n">
-        <v>445847.58</v>
+        <v>450064.38</v>
       </c>
       <c r="I89" s="4" t="n">
-        <v>22651.2</v>
+        <v>18434.4</v>
       </c>
       <c r="J89" s="5" t="n">
-        <v>0.0508</v>
+        <v>0.04099999999999999</v>
       </c>
       <c r="K89" t="inlineStr">
         <is>
@@ -5568,13 +5568,13 @@
         <v>0.0354</v>
       </c>
       <c r="H90" s="4" t="n">
-        <v>312996.64</v>
+        <v>323136.44</v>
       </c>
       <c r="I90" s="4" t="n">
-        <v>40127.35</v>
+        <v>29987.55</v>
       </c>
       <c r="J90" s="5" t="n">
-        <v>0.1282</v>
+        <v>0.09279999999999999</v>
       </c>
       <c r="K90" t="inlineStr">
         <is>
@@ -5621,13 +5621,13 @@
         <v>0.0102</v>
       </c>
       <c r="H91" s="4" t="n">
-        <v>349543.21</v>
+        <v>354590.53</v>
       </c>
       <c r="I91" s="4" t="n">
-        <v>40089.27</v>
+        <v>35041.95</v>
       </c>
       <c r="J91" s="5" t="n">
-        <v>0.1147</v>
+        <v>0.09880000000000001</v>
       </c>
       <c r="K91" t="inlineStr">
         <is>
@@ -5636,7 +5636,7 @@
       </c>
       <c r="L91" t="inlineStr">
         <is>
-          <t>Deviation</t>
+          <t>On Plan</t>
         </is>
       </c>
       <c r="M91" t="inlineStr">
@@ -5674,13 +5674,13 @@
         <v>-0.0312</v>
       </c>
       <c r="H92" s="4" t="n">
-        <v>399234.01</v>
+        <v>368127.22</v>
       </c>
       <c r="I92" s="4" t="n">
-        <v>13753.46</v>
+        <v>44860.25</v>
       </c>
       <c r="J92" s="5" t="n">
-        <v>0.0344</v>
+        <v>0.1219</v>
       </c>
       <c r="K92" t="inlineStr">
         <is>
@@ -5727,13 +5727,13 @@
         <v>-0.0362</v>
       </c>
       <c r="H93" s="4" t="n">
-        <v>840566.54</v>
+        <v>879627.86</v>
       </c>
       <c r="I93" s="4" t="n">
-        <v>88748.02</v>
+        <v>49686.7</v>
       </c>
       <c r="J93" s="5" t="n">
-        <v>0.1056</v>
+        <v>0.0565</v>
       </c>
       <c r="K93" t="inlineStr">
         <is>
@@ -5780,13 +5780,13 @@
         <v>0.0363</v>
       </c>
       <c r="H94" s="4" t="n">
-        <v>71211.78999999999</v>
+        <v>70940.50999999999</v>
       </c>
       <c r="I94" s="4" t="n">
-        <v>8065.56</v>
+        <v>8336.84</v>
       </c>
       <c r="J94" s="5" t="n">
-        <v>0.1133</v>
+        <v>0.1175</v>
       </c>
       <c r="K94" t="inlineStr">
         <is>
@@ -5833,13 +5833,13 @@
         <v>-0.0189</v>
       </c>
       <c r="H95" s="4" t="n">
-        <v>54088.03</v>
+        <v>56603.37</v>
       </c>
       <c r="I95" s="4" t="n">
-        <v>5953.52</v>
+        <v>3438.18</v>
       </c>
       <c r="J95" s="5" t="n">
-        <v>0.1101</v>
+        <v>0.0607</v>
       </c>
       <c r="K95" t="inlineStr">
         <is>
@@ -5848,7 +5848,7 @@
       </c>
       <c r="L95" t="inlineStr">
         <is>
-          <t>Deviation</t>
+          <t>On Plan</t>
         </is>
       </c>
       <c r="M95" t="inlineStr">
@@ -5886,13 +5886,13 @@
         <v>0.0301</v>
       </c>
       <c r="H96" s="4" t="n">
-        <v>40500.95</v>
+        <v>42028.26</v>
       </c>
       <c r="I96" s="4" t="n">
-        <v>6779.18</v>
+        <v>5251.87</v>
       </c>
       <c r="J96" s="5" t="n">
-        <v>0.1674</v>
+        <v>0.125</v>
       </c>
       <c r="K96" t="inlineStr">
         <is>
@@ -5939,13 +5939,13 @@
         <v>0.0023</v>
       </c>
       <c r="H97" s="4" t="n">
-        <v>212990.16</v>
+        <v>214806.99</v>
       </c>
       <c r="I97" s="4" t="n">
-        <v>29926.31</v>
+        <v>28109.48</v>
       </c>
       <c r="J97" s="5" t="n">
-        <v>0.1405</v>
+        <v>0.1309</v>
       </c>
       <c r="K97" t="inlineStr">
         <is>
@@ -5992,13 +5992,13 @@
         <v>0.0377</v>
       </c>
       <c r="H98" s="4" t="n">
-        <v>149804.05</v>
+        <v>152933.37</v>
       </c>
       <c r="I98" s="4" t="n">
-        <v>21663.23</v>
+        <v>18533.91</v>
       </c>
       <c r="J98" s="5" t="n">
-        <v>0.1446</v>
+        <v>0.1212</v>
       </c>
       <c r="K98" t="inlineStr">
         <is>
@@ -6045,13 +6045,13 @@
         <v>0.0397</v>
       </c>
       <c r="H99" s="4" t="n">
-        <v>291568.79</v>
+        <v>270186.16</v>
       </c>
       <c r="I99" s="4" t="n">
-        <v>29121.42</v>
+        <v>50504.05</v>
       </c>
       <c r="J99" s="5" t="n">
-        <v>0.0999</v>
+        <v>0.1869</v>
       </c>
       <c r="K99" t="inlineStr">
         <is>
@@ -6098,13 +6098,13 @@
         <v>0.0289</v>
       </c>
       <c r="H100" s="4" t="n">
-        <v>78562.64999999999</v>
+        <v>78527.2</v>
       </c>
       <c r="I100" s="4" t="n">
-        <v>12108.93</v>
+        <v>12144.38</v>
       </c>
       <c r="J100" s="5" t="n">
-        <v>0.1541</v>
+        <v>0.1547</v>
       </c>
       <c r="K100" t="inlineStr">
         <is>
@@ -6151,13 +6151,13 @@
         <v>0</v>
       </c>
       <c r="H101" s="4" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="I101" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J101" s="5" t="n">
-        <v>0.0741</v>
+        <v>0.1154</v>
       </c>
       <c r="K101" t="inlineStr">
         <is>
@@ -6204,13 +6204,13 @@
         <v>0</v>
       </c>
       <c r="H102" s="4" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="I102" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J102" s="5" t="n">
-        <v>0</v>
+        <v>0.09089999999999999</v>
       </c>
       <c r="K102" t="inlineStr">
         <is>
@@ -6363,13 +6363,13 @@
         <v>0.0177</v>
       </c>
       <c r="H105" s="4" t="n">
-        <v>119330.26</v>
+        <v>123189.6</v>
       </c>
       <c r="I105" s="4" t="n">
-        <v>15195.95</v>
+        <v>11336.61</v>
       </c>
       <c r="J105" s="5" t="n">
-        <v>0.1273</v>
+        <v>0.092</v>
       </c>
       <c r="K105" t="inlineStr">
         <is>
@@ -6416,13 +6416,13 @@
         <v>-0.0187</v>
       </c>
       <c r="H106" s="4" t="n">
-        <v>58282.08</v>
+        <v>56750.76</v>
       </c>
       <c r="I106" s="4" t="n">
-        <v>6580.97</v>
+        <v>8112.29</v>
       </c>
       <c r="J106" s="5" t="n">
-        <v>0.1129</v>
+        <v>0.1429</v>
       </c>
       <c r="K106" t="inlineStr">
         <is>
@@ -6469,13 +6469,13 @@
         <v>0.0145</v>
       </c>
       <c r="H107" s="4" t="n">
-        <v>92816.09</v>
+        <v>87208.71000000001</v>
       </c>
       <c r="I107" s="4" t="n">
-        <v>7769.15</v>
+        <v>13376.53</v>
       </c>
       <c r="J107" s="5" t="n">
-        <v>0.0837</v>
+        <v>0.1534</v>
       </c>
       <c r="K107" t="inlineStr">
         <is>
@@ -6522,13 +6522,13 @@
         <v>-0.0391</v>
       </c>
       <c r="H108" s="4" t="n">
-        <v>393496.39</v>
+        <v>387083.08</v>
       </c>
       <c r="I108" s="4" t="n">
-        <v>8751.77</v>
+        <v>15165.08</v>
       </c>
       <c r="J108" s="5" t="n">
-        <v>0.0222</v>
+        <v>0.0392</v>
       </c>
       <c r="K108" t="inlineStr">
         <is>
@@ -6575,13 +6575,13 @@
         <v>0.003</v>
       </c>
       <c r="H109" s="4" t="n">
-        <v>36041.94</v>
+        <v>33322.04</v>
       </c>
       <c r="I109" s="4" t="n">
-        <v>2628.09</v>
+        <v>5347.99</v>
       </c>
       <c r="J109" s="5" t="n">
-        <v>0.07290000000000001</v>
+        <v>0.1605</v>
       </c>
       <c r="K109" t="inlineStr">
         <is>
@@ -6628,13 +6628,13 @@
         <v>-0.0095</v>
       </c>
       <c r="H110" s="4" t="n">
-        <v>184834.47</v>
+        <v>176685.8</v>
       </c>
       <c r="I110" s="4" t="n">
-        <v>11575.65</v>
+        <v>19724.32</v>
       </c>
       <c r="J110" s="5" t="n">
-        <v>0.0626</v>
+        <v>0.1116</v>
       </c>
       <c r="K110" t="inlineStr">
         <is>
@@ -6681,13 +6681,13 @@
         <v>0.0234</v>
       </c>
       <c r="H111" s="4" t="n">
-        <v>812097.37</v>
+        <v>765922.48</v>
       </c>
       <c r="I111" s="4" t="n">
-        <v>89774.92999999999</v>
+        <v>135949.82</v>
       </c>
       <c r="J111" s="5" t="n">
-        <v>0.1105</v>
+        <v>0.1775</v>
       </c>
       <c r="K111" t="inlineStr">
         <is>
@@ -6734,13 +6734,13 @@
         <v>-0.0062</v>
       </c>
       <c r="H112" s="4" t="n">
-        <v>447516.69</v>
+        <v>445407.46</v>
       </c>
       <c r="I112" s="4" t="n">
-        <v>45116.36</v>
+        <v>47225.59</v>
       </c>
       <c r="J112" s="5" t="n">
-        <v>0.1008</v>
+        <v>0.106</v>
       </c>
       <c r="K112" t="inlineStr">
         <is>
@@ -6787,13 +6787,13 @@
         <v>-0.0349</v>
       </c>
       <c r="H113" s="4" t="n">
-        <v>310748</v>
+        <v>303653.21</v>
       </c>
       <c r="I113" s="4" t="n">
-        <v>29455.06</v>
+        <v>36549.85</v>
       </c>
       <c r="J113" s="5" t="n">
-        <v>0.09480000000000001</v>
+        <v>0.1204</v>
       </c>
       <c r="K113" t="inlineStr">
         <is>
@@ -6840,13 +6840,13 @@
         <v>0.033</v>
       </c>
       <c r="H114" s="4" t="n">
-        <v>349237.83</v>
+        <v>332832.49</v>
       </c>
       <c r="I114" s="4" t="n">
-        <v>51156.93</v>
+        <v>67562.27</v>
       </c>
       <c r="J114" s="5" t="n">
-        <v>0.1465</v>
+        <v>0.203</v>
       </c>
       <c r="K114" t="inlineStr">
         <is>
@@ -6893,13 +6893,13 @@
         <v>-0.0257</v>
       </c>
       <c r="H115" s="4" t="n">
-        <v>405677.59</v>
+        <v>374783.3</v>
       </c>
       <c r="I115" s="4" t="n">
-        <v>11709.17</v>
+        <v>42603.46</v>
       </c>
       <c r="J115" s="5" t="n">
-        <v>0.0289</v>
+        <v>0.1137</v>
       </c>
       <c r="K115" t="inlineStr">
         <is>
@@ -6946,13 +6946,13 @@
         <v>0</v>
       </c>
       <c r="H116" s="4" t="n">
-        <v>881598.36</v>
+        <v>913296.0699999999</v>
       </c>
       <c r="I116" s="4" t="n">
-        <v>87447.08</v>
+        <v>55749.37</v>
       </c>
       <c r="J116" s="5" t="n">
-        <v>0.0992</v>
+        <v>0.061</v>
       </c>
       <c r="K116" t="inlineStr">
         <is>
@@ -6961,7 +6961,7 @@
       </c>
       <c r="L116" t="inlineStr">
         <is>
-          <t>Deviation</t>
+          <t>On Plan</t>
         </is>
       </c>
       <c r="M116" t="inlineStr">
@@ -6999,13 +6999,13 @@
         <v>0.0302</v>
       </c>
       <c r="H117" s="4" t="n">
-        <v>70129.45</v>
+        <v>72161.39</v>
       </c>
       <c r="I117" s="4" t="n">
-        <v>9070.309999999999</v>
+        <v>7038.37</v>
       </c>
       <c r="J117" s="5" t="n">
-        <v>0.1293</v>
+        <v>0.0975</v>
       </c>
       <c r="K117" t="inlineStr">
         <is>
@@ -7052,13 +7052,13 @@
         <v>-0.0331</v>
       </c>
       <c r="H118" s="4" t="n">
-        <v>57854.12</v>
+        <v>56386.88</v>
       </c>
       <c r="I118" s="4" t="n">
-        <v>1607.29</v>
+        <v>3074.53</v>
       </c>
       <c r="J118" s="5" t="n">
-        <v>0.0278</v>
+        <v>0.0545</v>
       </c>
       <c r="K118" t="inlineStr">
         <is>
@@ -7105,13 +7105,13 @@
         <v>0.0358</v>
       </c>
       <c r="H119" s="4" t="n">
-        <v>42727.89</v>
+        <v>40972.15</v>
       </c>
       <c r="I119" s="4" t="n">
-        <v>5046.35</v>
+        <v>6802.09</v>
       </c>
       <c r="J119" s="5" t="n">
-        <v>0.1181</v>
+        <v>0.166</v>
       </c>
       <c r="K119" t="inlineStr">
         <is>
@@ -7158,13 +7158,13 @@
         <v>0.021</v>
       </c>
       <c r="H120" s="4" t="n">
-        <v>221645.79</v>
+        <v>227080.89</v>
       </c>
       <c r="I120" s="4" t="n">
-        <v>31613.47</v>
+        <v>26178.37</v>
       </c>
       <c r="J120" s="5" t="n">
-        <v>0.1426</v>
+        <v>0.1153</v>
       </c>
       <c r="K120" t="inlineStr">
         <is>
@@ -7211,13 +7211,13 @@
         <v>0.0032</v>
       </c>
       <c r="H121" s="4" t="n">
-        <v>149094.58</v>
+        <v>155851.51</v>
       </c>
       <c r="I121" s="4" t="n">
-        <v>20563.22</v>
+        <v>13806.29</v>
       </c>
       <c r="J121" s="5" t="n">
-        <v>0.1379</v>
+        <v>0.0886</v>
       </c>
       <c r="K121" t="inlineStr">
         <is>
@@ -7264,13 +7264,13 @@
         <v>-0.0278</v>
       </c>
       <c r="H122" s="4" t="n">
-        <v>284590.63</v>
+        <v>275368.24</v>
       </c>
       <c r="I122" s="4" t="n">
-        <v>22341.48</v>
+        <v>31563.87</v>
       </c>
       <c r="J122" s="5" t="n">
-        <v>0.0785</v>
+        <v>0.1146</v>
       </c>
       <c r="K122" t="inlineStr">
         <is>
@@ -7317,13 +7317,13 @@
         <v>0.0223</v>
       </c>
       <c r="H123" s="4" t="n">
-        <v>78439.33</v>
+        <v>78270.42</v>
       </c>
       <c r="I123" s="4" t="n">
-        <v>13771.24</v>
+        <v>13940.15</v>
       </c>
       <c r="J123" s="5" t="n">
-        <v>0.1756</v>
+        <v>0.1781</v>
       </c>
       <c r="K123" t="inlineStr">
         <is>
@@ -7370,13 +7370,13 @@
         <v>0.0345</v>
       </c>
       <c r="H124" s="4" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="I124" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J124" s="5" t="n">
-        <v>0.1538</v>
+        <v>0.2</v>
       </c>
       <c r="K124" t="inlineStr">
         <is>
@@ -7395,7 +7395,7 @@
       </c>
       <c r="N124" t="inlineStr">
         <is>
-          <t>Engineering headcount was 1 above plan in June 2024. This is a deviation from plan, flagged for routine review. Compared to the same period last year, this is up 15.4%.</t>
+          <t>Engineering headcount was 1 above plan in June 2024. This is a deviation from plan, flagged for routine review. Compared to the same period last year, this is up 20.0%.</t>
         </is>
       </c>
     </row>
@@ -7481,13 +7481,13 @@
         <v>0.0667</v>
       </c>
       <c r="H126" s="4" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="I126" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J126" s="5" t="n">
-        <v>0.1429</v>
+        <v>0.2308</v>
       </c>
       <c r="K126" t="inlineStr">
         <is>
@@ -7506,7 +7506,7 @@
       </c>
       <c r="N126" t="inlineStr">
         <is>
-          <t>Sales headcount was 1 above plan in June 2024. This is a deviation from plan, flagged for routine review. Compared to the same period last year, this is up 14.3%.</t>
+          <t>Sales headcount was 1 above plan in June 2024. This is a deviation from plan, flagged for routine review. Compared to the same period last year, this is up 23.1%.</t>
         </is>
       </c>
     </row>
@@ -7592,13 +7592,13 @@
         <v>-0.04</v>
       </c>
       <c r="H128" s="4" t="n">
-        <v>122311.91</v>
+        <v>124450.81</v>
       </c>
       <c r="I128" s="4" t="n">
-        <v>7582.28</v>
+        <v>5443.38</v>
       </c>
       <c r="J128" s="5" t="n">
-        <v>0.062</v>
+        <v>0.0437</v>
       </c>
       <c r="K128" t="inlineStr">
         <is>
@@ -7645,13 +7645,13 @@
         <v>0.0343</v>
       </c>
       <c r="H129" s="4" t="n">
-        <v>57949.03</v>
+        <v>63541.78</v>
       </c>
       <c r="I129" s="4" t="n">
-        <v>12023.25</v>
+        <v>6430.5</v>
       </c>
       <c r="J129" s="5" t="n">
-        <v>0.2075</v>
+        <v>0.1012</v>
       </c>
       <c r="K129" t="inlineStr">
         <is>
@@ -7698,13 +7698,13 @@
         <v>-0.0141</v>
       </c>
       <c r="H130" s="4" t="n">
-        <v>88653.28999999999</v>
+        <v>87569.17</v>
       </c>
       <c r="I130" s="4" t="n">
-        <v>11394.21</v>
+        <v>12478.33</v>
       </c>
       <c r="J130" s="5" t="n">
-        <v>0.1285</v>
+        <v>0.1425</v>
       </c>
       <c r="K130" t="inlineStr">
         <is>
@@ -7751,13 +7751,13 @@
         <v>0.0024</v>
       </c>
       <c r="H131" s="4" t="n">
-        <v>392155</v>
+        <v>388684.31</v>
       </c>
       <c r="I131" s="4" t="n">
-        <v>37335.4</v>
+        <v>40806.09</v>
       </c>
       <c r="J131" s="5" t="n">
-        <v>0.09519999999999999</v>
+        <v>0.105</v>
       </c>
       <c r="K131" t="inlineStr">
         <is>
@@ -7804,13 +7804,13 @@
         <v>-0.0384</v>
       </c>
       <c r="H132" s="4" t="n">
-        <v>36395.98</v>
+        <v>36550.96</v>
       </c>
       <c r="I132" s="4" t="n">
-        <v>1549.51</v>
+        <v>1394.53</v>
       </c>
       <c r="J132" s="5" t="n">
-        <v>0.0426</v>
+        <v>0.0382</v>
       </c>
       <c r="K132" t="inlineStr">
         <is>
@@ -7857,13 +7857,13 @@
         <v>0.008699999999999999</v>
       </c>
       <c r="H133" s="4" t="n">
-        <v>183105.73</v>
+        <v>183325.27</v>
       </c>
       <c r="I133" s="4" t="n">
-        <v>21613.51</v>
+        <v>21393.97</v>
       </c>
       <c r="J133" s="5" t="n">
-        <v>0.118</v>
+        <v>0.1167</v>
       </c>
       <c r="K133" t="inlineStr">
         <is>
@@ -7910,13 +7910,13 @@
         <v>0.0296</v>
       </c>
       <c r="H134" s="4" t="n">
-        <v>781150.29</v>
+        <v>781456.87</v>
       </c>
       <c r="I134" s="4" t="n">
-        <v>147586.33</v>
+        <v>147279.75</v>
       </c>
       <c r="J134" s="5" t="n">
-        <v>0.1889</v>
+        <v>0.1885</v>
       </c>
       <c r="K134" t="inlineStr">
         <is>
@@ -7963,13 +7963,13 @@
         <v>-0.0161</v>
       </c>
       <c r="H135" s="4" t="n">
-        <v>457156.96</v>
+        <v>438378.1</v>
       </c>
       <c r="I135" s="4" t="n">
-        <v>42036.91</v>
+        <v>60815.77</v>
       </c>
       <c r="J135" s="5" t="n">
-        <v>0.092</v>
+        <v>0.1387</v>
       </c>
       <c r="K135" t="inlineStr">
         <is>
@@ -8016,13 +8016,13 @@
         <v>-0.1689</v>
       </c>
       <c r="H136" s="4" t="n">
-        <v>318824.49</v>
+        <v>329327.76</v>
       </c>
       <c r="I136" s="4" t="n">
-        <v>-18957.85</v>
+        <v>-29461.12</v>
       </c>
       <c r="J136" s="5" t="n">
-        <v>-0.0595</v>
+        <v>-0.0895</v>
       </c>
       <c r="K136" t="inlineStr">
         <is>
@@ -8041,7 +8041,7 @@
       </c>
       <c r="N136" t="inlineStr">
         <is>
-          <t>Subscription Revenue revenue fell short of budget by ₹60,933 (16.9%) in June 2024. This is an unfavorable variance, flagged as high priority for review. Compared to the same period last year, this is down 6.0%.</t>
+          <t>Subscription Revenue revenue fell short of budget by ₹60,933 (16.9%) in June 2024. This is an unfavorable variance, flagged as high priority for review. Compared to the same period last year, this is down 8.9%.</t>
         </is>
       </c>
     </row>
@@ -8074,13 +8074,13 @@
         <v>0.0208</v>
       </c>
       <c r="H137" s="4" t="n">
-        <v>349680.1</v>
+        <v>354048.39</v>
       </c>
       <c r="I137" s="4" t="n">
-        <v>47940.26</v>
+        <v>43571.97</v>
       </c>
       <c r="J137" s="5" t="n">
-        <v>0.1371</v>
+        <v>0.1231</v>
       </c>
       <c r="K137" t="inlineStr">
         <is>
@@ -8127,13 +8127,13 @@
         <v>-0.0345</v>
       </c>
       <c r="H138" s="4" t="n">
-        <v>368510.44</v>
+        <v>393765.34</v>
       </c>
       <c r="I138" s="4" t="n">
-        <v>47153.24</v>
+        <v>21898.34</v>
       </c>
       <c r="J138" s="5" t="n">
-        <v>0.128</v>
+        <v>0.0556</v>
       </c>
       <c r="K138" t="inlineStr">
         <is>
@@ -8180,13 +8180,13 @@
         <v>-0.0011</v>
       </c>
       <c r="H139" s="4" t="n">
-        <v>873591.72</v>
+        <v>836942.09</v>
       </c>
       <c r="I139" s="4" t="n">
-        <v>99066.94</v>
+        <v>135716.57</v>
       </c>
       <c r="J139" s="5" t="n">
-        <v>0.1134</v>
+        <v>0.1622</v>
       </c>
       <c r="K139" t="inlineStr">
         <is>
@@ -8195,7 +8195,7 @@
       </c>
       <c r="L139" t="inlineStr">
         <is>
-          <t>Deviation</t>
+          <t>On Plan</t>
         </is>
       </c>
       <c r="M139" t="inlineStr">
@@ -8301,7 +8301,7 @@
       </c>
       <c r="L141" t="inlineStr">
         <is>
-          <t>Deviation</t>
+          <t>On Plan</t>
         </is>
       </c>
       <c r="M141" t="inlineStr">
@@ -8354,7 +8354,7 @@
       </c>
       <c r="L142" t="inlineStr">
         <is>
-          <t>Deviation</t>
+          <t>On Plan</t>
         </is>
       </c>
       <c r="M142" t="inlineStr">
@@ -9467,7 +9467,7 @@
       </c>
       <c r="L163" t="inlineStr">
         <is>
-          <t>Deviation</t>
+          <t>On Plan</t>
         </is>
       </c>
       <c r="M163" t="inlineStr">
@@ -9520,7 +9520,7 @@
       </c>
       <c r="L164" t="inlineStr">
         <is>
-          <t>Deviation</t>
+          <t>On Plan</t>
         </is>
       </c>
       <c r="M164" t="inlineStr">
@@ -9573,7 +9573,7 @@
       </c>
       <c r="L165" t="inlineStr">
         <is>
-          <t>Deviation</t>
+          <t>On Plan</t>
         </is>
       </c>
       <c r="M165" t="inlineStr">
@@ -10648,7 +10648,7 @@
       </c>
       <c r="L185" t="inlineStr">
         <is>
-          <t>Deviation</t>
+          <t>On Plan</t>
         </is>
       </c>
       <c r="M185" t="inlineStr">
@@ -11776,7 +11776,7 @@
       </c>
       <c r="L206" t="inlineStr">
         <is>
-          <t>Deviation</t>
+          <t>On Plan</t>
         </is>
       </c>
       <c r="M206" t="inlineStr">
@@ -11882,7 +11882,7 @@
       </c>
       <c r="L208" t="inlineStr">
         <is>
-          <t>Deviation</t>
+          <t>On Plan</t>
         </is>
       </c>
       <c r="M208" t="inlineStr">
@@ -11988,7 +11988,7 @@
       </c>
       <c r="L210" t="inlineStr">
         <is>
-          <t>Deviation</t>
+          <t>On Plan</t>
         </is>
       </c>
       <c r="M210" t="inlineStr">
@@ -12041,7 +12041,7 @@
       </c>
       <c r="L211" t="inlineStr">
         <is>
-          <t>Deviation</t>
+          <t>On Plan</t>
         </is>
       </c>
       <c r="M211" t="inlineStr">
@@ -13164,7 +13164,7 @@
       </c>
       <c r="L232" t="inlineStr">
         <is>
-          <t>Deviation</t>
+          <t>On Plan</t>
         </is>
       </c>
       <c r="M232" t="inlineStr">
@@ -13217,7 +13217,7 @@
       </c>
       <c r="L233" t="inlineStr">
         <is>
-          <t>Deviation</t>
+          <t>On Plan</t>
         </is>
       </c>
       <c r="M233" t="inlineStr">
@@ -13270,7 +13270,7 @@
       </c>
       <c r="L234" t="inlineStr">
         <is>
-          <t>Deviation</t>
+          <t>On Plan</t>
         </is>
       </c>
       <c r="M234" t="inlineStr">
@@ -14345,7 +14345,7 @@
       </c>
       <c r="L254" t="inlineStr">
         <is>
-          <t>Deviation</t>
+          <t>On Plan</t>
         </is>
       </c>
       <c r="M254" t="inlineStr">
@@ -14451,7 +14451,7 @@
       </c>
       <c r="L256" t="inlineStr">
         <is>
-          <t>Deviation</t>
+          <t>On Plan</t>
         </is>
       </c>
       <c r="M256" t="inlineStr">
@@ -14504,7 +14504,7 @@
       </c>
       <c r="L257" t="inlineStr">
         <is>
-          <t>Deviation</t>
+          <t>On Plan</t>
         </is>
       </c>
       <c r="M257" t="inlineStr">
@@ -15622,7 +15622,7 @@
       </c>
       <c r="L278" t="inlineStr">
         <is>
-          <t>Deviation</t>
+          <t>On Plan</t>
         </is>
       </c>
       <c r="M278" t="inlineStr">
@@ -15675,7 +15675,7 @@
       </c>
       <c r="L279" t="inlineStr">
         <is>
-          <t>Deviation</t>
+          <t>On Plan</t>
         </is>
       </c>
       <c r="M279" t="inlineStr">
@@ -15728,7 +15728,7 @@
       </c>
       <c r="L280" t="inlineStr">
         <is>
-          <t>Deviation</t>
+          <t>On Plan</t>
         </is>
       </c>
       <c r="M280" t="inlineStr">
@@ -16788,7 +16788,7 @@
       </c>
       <c r="L300" t="inlineStr">
         <is>
-          <t>Deviation</t>
+          <t>On Plan</t>
         </is>
       </c>
       <c r="M300" t="inlineStr">
@@ -16841,7 +16841,7 @@
       </c>
       <c r="L301" t="inlineStr">
         <is>
-          <t>Deviation</t>
+          <t>On Plan</t>
         </is>
       </c>
       <c r="M301" t="inlineStr">
@@ -16947,7 +16947,7 @@
       </c>
       <c r="L303" t="inlineStr">
         <is>
-          <t>Deviation</t>
+          <t>On Plan</t>
         </is>
       </c>
       <c r="M303" t="inlineStr">
@@ -18060,7 +18060,7 @@
       </c>
       <c r="L324" t="inlineStr">
         <is>
-          <t>Deviation</t>
+          <t>On Plan</t>
         </is>
       </c>
       <c r="M324" t="inlineStr">
@@ -19125,7 +19125,7 @@
       </c>
       <c r="L344" t="inlineStr">
         <is>
-          <t>Deviation</t>
+          <t>On Plan</t>
         </is>
       </c>
       <c r="M344" t="inlineStr">
@@ -19284,7 +19284,7 @@
       </c>
       <c r="L347" t="inlineStr">
         <is>
-          <t>Deviation</t>
+          <t>On Plan</t>
         </is>
       </c>
       <c r="M347" t="inlineStr">
@@ -19337,7 +19337,7 @@
       </c>
       <c r="L348" t="inlineStr">
         <is>
-          <t>Deviation</t>
+          <t>On Plan</t>
         </is>
       </c>
       <c r="M348" t="inlineStr">
@@ -19390,7 +19390,7 @@
       </c>
       <c r="L349" t="inlineStr">
         <is>
-          <t>Deviation</t>
+          <t>On Plan</t>
         </is>
       </c>
       <c r="M349" t="inlineStr">
@@ -20349,7 +20349,7 @@
       </c>
       <c r="L367" t="inlineStr">
         <is>
-          <t>Deviation</t>
+          <t>On Plan</t>
         </is>
       </c>
       <c r="M367" t="inlineStr">
@@ -20402,7 +20402,7 @@
       </c>
       <c r="L368" t="inlineStr">
         <is>
-          <t>Deviation</t>
+          <t>On Plan</t>
         </is>
       </c>
       <c r="M368" t="inlineStr">
@@ -20455,7 +20455,7 @@
       </c>
       <c r="L369" t="inlineStr">
         <is>
-          <t>Deviation</t>
+          <t>On Plan</t>
         </is>
       </c>
       <c r="M369" t="inlineStr">
@@ -20508,7 +20508,7 @@
       </c>
       <c r="L370" t="inlineStr">
         <is>
-          <t>Deviation</t>
+          <t>On Plan</t>
         </is>
       </c>
       <c r="M370" t="inlineStr">
@@ -20561,7 +20561,7 @@
       </c>
       <c r="L371" t="inlineStr">
         <is>
-          <t>Deviation</t>
+          <t>On Plan</t>
         </is>
       </c>
       <c r="M371" t="inlineStr">
@@ -21626,7 +21626,7 @@
       </c>
       <c r="L391" t="inlineStr">
         <is>
-          <t>Deviation</t>
+          <t>On Plan</t>
         </is>
       </c>
       <c r="M391" t="inlineStr">
@@ -21732,7 +21732,7 @@
       </c>
       <c r="L393" t="inlineStr">
         <is>
-          <t>Deviation</t>
+          <t>On Plan</t>
         </is>
       </c>
       <c r="M393" t="inlineStr">
@@ -21838,7 +21838,7 @@
       </c>
       <c r="L395" t="inlineStr">
         <is>
-          <t>Deviation</t>
+          <t>On Plan</t>
         </is>
       </c>
       <c r="M395" t="inlineStr">
@@ -22855,7 +22855,7 @@
       </c>
       <c r="L414" t="inlineStr">
         <is>
-          <t>Deviation</t>
+          <t>On Plan</t>
         </is>
       </c>
       <c r="M414" t="inlineStr">

</xml_diff>

<commit_message>
Correct README findings and regenerate sample output
Findings, stage table and design notes now match what the pipeline
produces; sample_output regenerated from the fixed code.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/sample_output/variance_report.xlsx
+++ b/sample_output/variance_report.xlsx
@@ -101,9 +101,9 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -515,7 +515,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:F20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -634,8 +634,8 @@
       <c r="E7" s="5" t="n">
         <v>0.00505902192242833</v>
       </c>
-      <c r="F7" s="6" t="n">
-        <v>20</v>
+      <c r="F7" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -707,7 +707,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Favorable vs Unfavorable (All Items)</t>
+          <t>Variance Status (All Items)</t>
         </is>
       </c>
     </row>
@@ -718,28 +718,48 @@
         </is>
       </c>
       <c r="B14" s="7" t="n">
-        <v>161</v>
+        <v>109</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
+          <t>On Plan</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
           <t>Unfavorable</t>
         </is>
       </c>
-      <c r="B15" s="8" t="n">
-        <v>253</v>
+      <c r="B16" s="8" t="n">
+        <v>125</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="inlineStr">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Deviation</t>
+        </is>
+      </c>
+      <c r="B17" s="9" t="n">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
         <is>
           <t>High-Risk Material Variances</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="6" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="6" t="inlineStr">
         <is>
           <t>3 item(s) flagged HIGH risk - see 'Flagged' tab</t>
         </is>
@@ -1260,7 +1280,7 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -1271,11 +1291,6 @@
       <c r="M9" t="inlineStr">
         <is>
           <t>MEDIUM</t>
-        </is>
-      </c>
-      <c r="N9" t="inlineStr">
-        <is>
-          <t>Engineering headcount was 1 below plan in January 2024. This is a deviation from plan, flagged for routine review. Compared to the same period last year, this is up 12.5%.</t>
         </is>
       </c>
     </row>
@@ -2484,7 +2499,7 @@
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
@@ -2495,11 +2510,6 @@
       <c r="M32" t="inlineStr">
         <is>
           <t>MEDIUM</t>
-        </is>
-      </c>
-      <c r="N32" t="inlineStr">
-        <is>
-          <t>Engineering headcount was 1 above plan in February 2024. This is a deviation from plan, flagged for routine review. Compared to the same period last year, this is up 7.4%.</t>
         </is>
       </c>
     </row>
@@ -3814,7 +3824,7 @@
       </c>
       <c r="K57" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="L57" t="inlineStr">
@@ -3825,11 +3835,6 @@
       <c r="M57" t="inlineStr">
         <is>
           <t>MEDIUM</t>
-        </is>
-      </c>
-      <c r="N57" t="inlineStr">
-        <is>
-          <t>Sales headcount was 1 above plan in March 2024. This is a deviation from plan, flagged for routine review. Compared to the same period last year, this is up 14.3%.</t>
         </is>
       </c>
     </row>
@@ -4932,7 +4937,7 @@
       </c>
       <c r="K78" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="L78" t="inlineStr">
@@ -4943,11 +4948,6 @@
       <c r="M78" t="inlineStr">
         <is>
           <t>MEDIUM</t>
-        </is>
-      </c>
-      <c r="N78" t="inlineStr">
-        <is>
-          <t>Engineering headcount was 1 above plan in April 2024. This is a deviation from plan, flagged for routine review. Compared to the same period last year, this is up 11.5%.</t>
         </is>
       </c>
     </row>
@@ -5043,7 +5043,7 @@
       </c>
       <c r="K80" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="L80" t="inlineStr">
@@ -5054,11 +5054,6 @@
       <c r="M80" t="inlineStr">
         <is>
           <t>MEDIUM</t>
-        </is>
-      </c>
-      <c r="N80" t="inlineStr">
-        <is>
-          <t>Sales headcount was 1 above plan in April 2024. This is a deviation from plan, flagged for routine review. Compared to the same period last year, this is up 23.1%.</t>
         </is>
       </c>
     </row>
@@ -7380,7 +7375,7 @@
       </c>
       <c r="K124" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="L124" t="inlineStr">
@@ -7391,11 +7386,6 @@
       <c r="M124" t="inlineStr">
         <is>
           <t>MEDIUM</t>
-        </is>
-      </c>
-      <c r="N124" t="inlineStr">
-        <is>
-          <t>Engineering headcount was 1 above plan in June 2024. This is a deviation from plan, flagged for routine review. Compared to the same period last year, this is up 20.0%.</t>
         </is>
       </c>
     </row>
@@ -7491,7 +7481,7 @@
       </c>
       <c r="K126" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="L126" t="inlineStr">
@@ -7502,11 +7492,6 @@
       <c r="M126" t="inlineStr">
         <is>
           <t>MEDIUM</t>
-        </is>
-      </c>
-      <c r="N126" t="inlineStr">
-        <is>
-          <t>Sales headcount was 1 above plan in June 2024. This is a deviation from plan, flagged for routine review. Compared to the same period last year, this is up 23.1%.</t>
         </is>
       </c>
     </row>
@@ -9833,7 +9818,7 @@
       </c>
       <c r="K170" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="L170" t="inlineStr">
@@ -9844,11 +9829,6 @@
       <c r="M170" t="inlineStr">
         <is>
           <t>MEDIUM</t>
-        </is>
-      </c>
-      <c r="N170" t="inlineStr">
-        <is>
-          <t>Engineering headcount was 1 above plan in August 2024. This is a deviation from plan, flagged for routine review. Compared to the same period last year, this is up 20.0%.</t>
         </is>
       </c>
     </row>
@@ -9944,7 +9924,7 @@
       </c>
       <c r="K172" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="L172" t="inlineStr">
@@ -9955,11 +9935,6 @@
       <c r="M172" t="inlineStr">
         <is>
           <t>MEDIUM</t>
-        </is>
-      </c>
-      <c r="N172" t="inlineStr">
-        <is>
-          <t>Sales headcount was 1 below plan in August 2024. This is a deviation from plan, flagged for routine review. Compared to the same period last year, this is up 15.4%.</t>
         </is>
       </c>
     </row>
@@ -11067,7 +11042,7 @@
       </c>
       <c r="K193" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="L193" t="inlineStr">
@@ -11078,11 +11053,6 @@
       <c r="M193" t="inlineStr">
         <is>
           <t>MEDIUM</t>
-        </is>
-      </c>
-      <c r="N193" t="inlineStr">
-        <is>
-          <t>Engineering headcount was 1 below plan in September 2024. This is a deviation from plan, flagged for routine review. Compared to the same period last year, this is up 12.0%.</t>
         </is>
       </c>
     </row>
@@ -11125,7 +11095,7 @@
       </c>
       <c r="K194" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="L194" t="inlineStr">
@@ -11136,11 +11106,6 @@
       <c r="M194" t="inlineStr">
         <is>
           <t>MEDIUM</t>
-        </is>
-      </c>
-      <c r="N194" t="inlineStr">
-        <is>
-          <t>Operations headcount was 1 above plan in September 2024. This is a deviation from plan, flagged for routine review. Compared to the same period last year, this is up 18.2%.</t>
         </is>
       </c>
     </row>
@@ -11236,7 +11201,7 @@
       </c>
       <c r="K196" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="L196" t="inlineStr">
@@ -11247,11 +11212,6 @@
       <c r="M196" t="inlineStr">
         <is>
           <t>MEDIUM</t>
-        </is>
-      </c>
-      <c r="N196" t="inlineStr">
-        <is>
-          <t>Support headcount was 1 above plan in September 2024. This is a deviation from plan, flagged for routine review. Compared to the same period last year, this is up 28.6%.</t>
         </is>
       </c>
     </row>
@@ -12301,7 +12261,7 @@
       </c>
       <c r="K216" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="L216" t="inlineStr">
@@ -12312,11 +12272,6 @@
       <c r="M216" t="inlineStr">
         <is>
           <t>MEDIUM</t>
-        </is>
-      </c>
-      <c r="N216" t="inlineStr">
-        <is>
-          <t>Engineering headcount was 1 above plan in October 2024. This is a deviation from plan, flagged for routine review. Compared to the same period last year, this is up 20.0%.</t>
         </is>
       </c>
     </row>
@@ -12465,7 +12420,7 @@
       </c>
       <c r="K219" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="L219" t="inlineStr">
@@ -12476,11 +12431,6 @@
       <c r="M219" t="inlineStr">
         <is>
           <t>MEDIUM</t>
-        </is>
-      </c>
-      <c r="N219" t="inlineStr">
-        <is>
-          <t>Support headcount was 1 above plan in October 2024. This is a deviation from plan, flagged for routine review. Compared to the same period last year, this is up 28.6%.</t>
         </is>
       </c>
     </row>
@@ -13535,7 +13485,7 @@
       </c>
       <c r="K239" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="L239" t="inlineStr">
@@ -13546,11 +13496,6 @@
       <c r="M239" t="inlineStr">
         <is>
           <t>MEDIUM</t>
-        </is>
-      </c>
-      <c r="N239" t="inlineStr">
-        <is>
-          <t>Engineering headcount was 1 above plan in November 2024. This is a deviation from plan, flagged for routine review. Compared to the same period last year, this is up 15.4%.</t>
         </is>
       </c>
     </row>
@@ -13646,7 +13591,7 @@
       </c>
       <c r="K241" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="L241" t="inlineStr">
@@ -13657,11 +13602,6 @@
       <c r="M241" t="inlineStr">
         <is>
           <t>MEDIUM</t>
-        </is>
-      </c>
-      <c r="N241" t="inlineStr">
-        <is>
-          <t>Sales headcount was 1 below plan in November 2024. This is a deviation from plan, flagged for routine review. Compared to the same period last year, this is up 15.4%.</t>
         </is>
       </c>
     </row>
@@ -19650,7 +19590,7 @@
       </c>
       <c r="K354" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="L354" t="inlineStr">
@@ -19661,11 +19601,6 @@
       <c r="M354" t="inlineStr">
         <is>
           <t>MEDIUM</t>
-        </is>
-      </c>
-      <c r="N354" t="inlineStr">
-        <is>
-          <t>Engineering headcount was 1 below plan in April 2025. This is a deviation from plan, flagged for routine review. Compared to the same period last year, this is up 20.0%.</t>
         </is>
       </c>
     </row>
@@ -20874,7 +20809,7 @@
       </c>
       <c r="K377" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="L377" t="inlineStr">
@@ -20885,11 +20820,6 @@
       <c r="M377" t="inlineStr">
         <is>
           <t>MEDIUM</t>
-        </is>
-      </c>
-      <c r="N377" t="inlineStr">
-        <is>
-          <t>Engineering headcount was 1 below plan in May 2025. This is a deviation from plan, flagged for routine review. Compared to the same period last year, this is up 11.1%.</t>
         </is>
       </c>
     </row>
@@ -22098,7 +22028,7 @@
       </c>
       <c r="K400" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="L400" t="inlineStr">
@@ -22109,11 +22039,6 @@
       <c r="M400" t="inlineStr">
         <is>
           <t>MEDIUM</t>
-        </is>
-      </c>
-      <c r="N400" t="inlineStr">
-        <is>
-          <t>Engineering headcount was 1 above plan in June 2025. This is a deviation from plan, flagged for routine review. Compared to the same period last year, this is up 23.1%.</t>
         </is>
       </c>
     </row>
@@ -22209,7 +22134,7 @@
       </c>
       <c r="K402" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="L402" t="inlineStr">
@@ -22220,11 +22145,6 @@
       <c r="M402" t="inlineStr">
         <is>
           <t>MEDIUM</t>
-        </is>
-      </c>
-      <c r="N402" t="inlineStr">
-        <is>
-          <t>Sales headcount was 1 below plan in June 2025. This is a deviation from plan, flagged for routine review. Compared to the same period last year, this is up 14.3%.</t>
         </is>
       </c>
     </row>
@@ -22942,7 +22862,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H28"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -23026,13 +22946,13 @@
       <c r="E4" s="4" t="n">
         <v>648574.79</v>
       </c>
-      <c r="F4" s="9" t="n">
+      <c r="F4" s="10" t="n">
         <v>-204265.21</v>
       </c>
       <c r="G4" s="5" t="n">
         <v>-0.2395</v>
       </c>
-      <c r="H4" s="10" t="inlineStr">
+      <c r="H4" s="11" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
@@ -23060,13 +22980,13 @@
       <c r="E5" s="4" t="n">
         <v>450585.35</v>
       </c>
-      <c r="F5" s="9" t="n">
+      <c r="F5" s="10" t="n">
         <v>103665.35</v>
       </c>
       <c r="G5" s="5" t="n">
         <v>0.2988</v>
       </c>
-      <c r="H5" s="10" t="inlineStr">
+      <c r="H5" s="11" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
@@ -23094,13 +23014,13 @@
       <c r="E6" s="4" t="n">
         <v>299866.64</v>
       </c>
-      <c r="F6" s="9" t="n">
+      <c r="F6" s="10" t="n">
         <v>-60933.36</v>
       </c>
       <c r="G6" s="5" t="n">
         <v>-0.1689</v>
       </c>
-      <c r="H6" s="10" t="inlineStr">
+      <c r="H6" s="11" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
@@ -23128,13 +23048,13 @@
       <c r="E7" s="4" t="n">
         <v>190964.25</v>
       </c>
-      <c r="F7" s="9" t="n">
+      <c r="F7" s="10" t="n">
         <v>57548.25</v>
       </c>
       <c r="G7" s="5" t="n">
         <v>0.4313</v>
       </c>
-      <c r="H7" s="11" t="inlineStr">
+      <c r="H7" s="9" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
@@ -23162,693 +23082,13 @@
       <c r="E8" s="4" t="n">
         <v>123932.16</v>
       </c>
-      <c r="F8" s="9" t="n">
+      <c r="F8" s="10" t="n">
         <v>44807.16</v>
       </c>
       <c r="G8" s="5" t="n">
         <v>0.5663</v>
       </c>
-      <c r="H8" s="11" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>2024-01</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Headcount</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>engineering</t>
-        </is>
-      </c>
-      <c r="D9" s="4" t="n">
-        <v>28</v>
-      </c>
-      <c r="E9" s="4" t="n">
-        <v>27</v>
-      </c>
-      <c r="F9" s="9" t="n">
-        <v>-1</v>
-      </c>
-      <c r="G9" s="5" t="n">
-        <v>-0.0357</v>
-      </c>
-      <c r="H9" s="11" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>2024-02</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Headcount</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>engineering</t>
-        </is>
-      </c>
-      <c r="D10" s="4" t="n">
-        <v>28</v>
-      </c>
-      <c r="E10" s="4" t="n">
-        <v>29</v>
-      </c>
-      <c r="F10" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="G10" s="5" t="n">
-        <v>0.0357</v>
-      </c>
-      <c r="H10" s="11" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>2024-03</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Headcount</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>sales</t>
-        </is>
-      </c>
-      <c r="D11" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="E11" s="4" t="n">
-        <v>16</v>
-      </c>
-      <c r="F11" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="G11" s="5" t="n">
-        <v>0.0667</v>
-      </c>
-      <c r="H11" s="11" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>2024-04</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Headcount</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>engineering</t>
-        </is>
-      </c>
-      <c r="D12" s="4" t="n">
-        <v>28</v>
-      </c>
-      <c r="E12" s="4" t="n">
-        <v>29</v>
-      </c>
-      <c r="F12" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="G12" s="5" t="n">
-        <v>0.0357</v>
-      </c>
-      <c r="H12" s="11" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>2024-04</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Headcount</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>sales</t>
-        </is>
-      </c>
-      <c r="D13" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="E13" s="4" t="n">
-        <v>16</v>
-      </c>
-      <c r="F13" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="G13" s="5" t="n">
-        <v>0.0667</v>
-      </c>
-      <c r="H13" s="11" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>2024-06</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Headcount</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>engineering</t>
-        </is>
-      </c>
-      <c r="D14" s="4" t="n">
-        <v>29</v>
-      </c>
-      <c r="E14" s="4" t="n">
-        <v>30</v>
-      </c>
-      <c r="F14" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="G14" s="5" t="n">
-        <v>0.0345</v>
-      </c>
-      <c r="H14" s="11" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>2024-06</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Headcount</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>sales</t>
-        </is>
-      </c>
-      <c r="D15" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="E15" s="4" t="n">
-        <v>16</v>
-      </c>
-      <c r="F15" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="G15" s="5" t="n">
-        <v>0.0667</v>
-      </c>
-      <c r="H15" s="11" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>2024-08</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Headcount</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>engineering</t>
-        </is>
-      </c>
-      <c r="D16" s="4" t="n">
-        <v>29</v>
-      </c>
-      <c r="E16" s="4" t="n">
-        <v>30</v>
-      </c>
-      <c r="F16" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="G16" s="5" t="n">
-        <v>0.0345</v>
-      </c>
-      <c r="H16" s="11" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>2024-08</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Headcount</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>sales</t>
-        </is>
-      </c>
-      <c r="D17" s="4" t="n">
-        <v>16</v>
-      </c>
-      <c r="E17" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="F17" s="9" t="n">
-        <v>-1</v>
-      </c>
-      <c r="G17" s="5" t="n">
-        <v>-0.0625</v>
-      </c>
-      <c r="H17" s="11" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>2024-09</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Headcount</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>engineering</t>
-        </is>
-      </c>
-      <c r="D18" s="4" t="n">
-        <v>29</v>
-      </c>
-      <c r="E18" s="4" t="n">
-        <v>28</v>
-      </c>
-      <c r="F18" s="9" t="n">
-        <v>-1</v>
-      </c>
-      <c r="G18" s="5" t="n">
-        <v>-0.0345</v>
-      </c>
-      <c r="H18" s="11" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>2024-09</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Headcount</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>operations</t>
-        </is>
-      </c>
-      <c r="D19" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="E19" s="4" t="n">
-        <v>13</v>
-      </c>
-      <c r="F19" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="G19" s="5" t="n">
-        <v>0.0833</v>
-      </c>
-      <c r="H19" s="11" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>2024-09</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Headcount</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>support</t>
-        </is>
-      </c>
-      <c r="D20" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="E20" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="F20" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="G20" s="5" t="n">
-        <v>0.125</v>
-      </c>
-      <c r="H20" s="11" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>2024-10</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Headcount</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>engineering</t>
-        </is>
-      </c>
-      <c r="D21" s="4" t="n">
-        <v>29</v>
-      </c>
-      <c r="E21" s="4" t="n">
-        <v>30</v>
-      </c>
-      <c r="F21" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="G21" s="5" t="n">
-        <v>0.0345</v>
-      </c>
-      <c r="H21" s="11" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>2024-10</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>Headcount</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>support</t>
-        </is>
-      </c>
-      <c r="D22" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="E22" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="F22" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="G22" s="5" t="n">
-        <v>0.125</v>
-      </c>
-      <c r="H22" s="11" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>2024-11</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Headcount</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>engineering</t>
-        </is>
-      </c>
-      <c r="D23" s="4" t="n">
-        <v>29</v>
-      </c>
-      <c r="E23" s="4" t="n">
-        <v>30</v>
-      </c>
-      <c r="F23" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="G23" s="5" t="n">
-        <v>0.0345</v>
-      </c>
-      <c r="H23" s="11" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>2024-11</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>Headcount</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>sales</t>
-        </is>
-      </c>
-      <c r="D24" s="4" t="n">
-        <v>16</v>
-      </c>
-      <c r="E24" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="F24" s="9" t="n">
-        <v>-1</v>
-      </c>
-      <c r="G24" s="5" t="n">
-        <v>-0.0625</v>
-      </c>
-      <c r="H24" s="11" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>2025-04</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>Headcount</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>engineering</t>
-        </is>
-      </c>
-      <c r="D25" s="4" t="n">
-        <v>31</v>
-      </c>
-      <c r="E25" s="4" t="n">
-        <v>30</v>
-      </c>
-      <c r="F25" s="9" t="n">
-        <v>-1</v>
-      </c>
-      <c r="G25" s="5" t="n">
-        <v>-0.0323</v>
-      </c>
-      <c r="H25" s="11" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>2025-05</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>Headcount</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>engineering</t>
-        </is>
-      </c>
-      <c r="D26" s="4" t="n">
-        <v>31</v>
-      </c>
-      <c r="E26" s="4" t="n">
-        <v>30</v>
-      </c>
-      <c r="F26" s="9" t="n">
-        <v>-1</v>
-      </c>
-      <c r="G26" s="5" t="n">
-        <v>-0.0323</v>
-      </c>
-      <c r="H26" s="11" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>2025-06</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>Headcount</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>engineering</t>
-        </is>
-      </c>
-      <c r="D27" s="4" t="n">
-        <v>31</v>
-      </c>
-      <c r="E27" s="4" t="n">
-        <v>32</v>
-      </c>
-      <c r="F27" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="G27" s="5" t="n">
-        <v>0.0323</v>
-      </c>
-      <c r="H27" s="11" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>2025-06</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>Headcount</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>sales</t>
-        </is>
-      </c>
-      <c r="D28" s="4" t="n">
-        <v>17</v>
-      </c>
-      <c r="E28" s="4" t="n">
-        <v>16</v>
-      </c>
-      <c r="F28" s="9" t="n">
-        <v>-1</v>
-      </c>
-      <c r="G28" s="5" t="n">
-        <v>-0.0588</v>
-      </c>
-      <c r="H28" s="11" t="inlineStr">
+      <c r="H8" s="9" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>

</xml_diff>